<commit_message>
Redraw Street Child and NRC after their accessibility updates (frame only)
On Jack's go. NRC's 21 Sep report merged (14 clusters newly inaccessible);
Street Child's two Madagali ward flips already in its returned file.
Accessibility chain refreshed, WORKING refreshed, then 8 clusters drawn with
the fixed draw and merged: Gwoza and Konduga back to Representative (9.93,
9.70); Madagali Non-IDP 18.76 -> 16.82, still not recoverable (1 of 11
clusters buildable). Partner packages deferred per Jack.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resampling/input/accessibility_reports_returned/NRC_accessibility_report.xlsx
+++ b/resampling/input/accessibility_reports_returned/NRC_accessibility_report.xlsx
@@ -28108,6 +28108,11 @@
           <t>12</t>
         </is>
       </c>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -28330,6 +28335,11 @@
           <t>36</t>
         </is>
       </c>
+      <c r="I225" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -29051,6 +29061,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I243" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -29604,6 +29619,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I257" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -29789,6 +29809,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I262" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -32980,6 +33005,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
@@ -33054,6 +33084,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -33091,6 +33126,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -33128,6 +33168,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -33165,6 +33210,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -33202,6 +33252,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -33350,6 +33405,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I355" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
@@ -33387,6 +33447,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I356" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -33424,6 +33489,11 @@
           <t>6</t>
         </is>
       </c>
+      <c r="I357" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -38721,7 +38791,6 @@
           <t>non_idp_NG002009_supp5</t>
         </is>
       </c>
-      <c r="F488" t="inlineStr"/>
       <c r="G488" t="inlineStr">
         <is>
           <t>6</t>
@@ -38759,7 +38828,6 @@
           <t>non_idp_NG008011_supp9</t>
         </is>
       </c>
-      <c r="F489" t="inlineStr"/>
       <c r="G489" t="inlineStr">
         <is>
           <t>6</t>
@@ -38797,7 +38865,6 @@
           <t>non_idp_NG008011_supp10</t>
         </is>
       </c>
-      <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr">
         <is>
           <t>6</t>
@@ -38835,7 +38902,6 @@
           <t>non_idp_NG008016_supp6</t>
         </is>
       </c>
-      <c r="F491" t="inlineStr"/>
       <c r="G491" t="inlineStr">
         <is>
           <t>6</t>

</xml_diff>